<commit_message>
Fix status change active to left & left to active timeout and handle popup with count validation
</commit_message>
<xml_diff>
--- a/features/testdata/contractor_employee.xlsx
+++ b/features/testdata/contractor_employee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CLMS-Automation\testing-framework-playwright--simplecode\features\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C392D54D-9E13-4DC0-A408-2A4B5E879C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2032652E-171D-4A28-A574-054677BC1439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="202">
   <si>
     <t>EmployeeCode</t>
   </si>
@@ -571,6 +571,66 @@
   </si>
   <si>
     <t>B</t>
+  </si>
+  <si>
+    <t>Rohit</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Mangal</t>
+  </si>
+  <si>
+    <t>Raval</t>
+  </si>
+  <si>
+    <t>Swati</t>
+  </si>
+  <si>
+    <t>Bondre</t>
+  </si>
+  <si>
+    <t>Manish</t>
+  </si>
+  <si>
+    <t>Mandavkar</t>
+  </si>
+  <si>
+    <t>Waghare</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Prabhat</t>
+  </si>
+  <si>
+    <t>Umesh</t>
+  </si>
+  <si>
+    <t>Garware</t>
+  </si>
+  <si>
+    <t>Devika</t>
+  </si>
+  <si>
+    <t>Malkhabe</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>AB+</t>
+  </si>
+  <si>
+    <t>O+</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Left</t>
   </si>
 </sst>
 </file>
@@ -613,11 +673,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -648,7 +710,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ContratorEmployee" displayName="ContratorEmployee" ref="A1:EV3" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ContratorEmployee" displayName="ContratorEmployee" ref="A1:EV13" totalsRowShown="0">
   <tableColumns count="152">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="EmployeeCode"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="FirstName"/>
@@ -1092,7 +1154,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EV3"/>
+  <dimension ref="A1:EV13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" customWidth="1"/>
@@ -1905,7 +1967,10 @@
         <v>154</v>
       </c>
       <c r="J3" t="s">
-        <v>156</v>
+        <v>198</v>
+      </c>
+      <c r="K3" t="s">
+        <v>157</v>
       </c>
       <c r="M3" t="s">
         <v>158</v>
@@ -1968,6 +2033,507 @@
       <c r="BQ3" s="3">
         <v>961201180204</v>
       </c>
+    </row>
+    <row r="4" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>556700</v>
+      </c>
+      <c r="B4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D4" t="s">
+        <v>191</v>
+      </c>
+      <c r="G4" s="5">
+        <v>32831</v>
+      </c>
+      <c r="H4" t="s">
+        <v>154</v>
+      </c>
+      <c r="J4" t="s">
+        <v>156</v>
+      </c>
+      <c r="K4" t="s">
+        <v>157</v>
+      </c>
+      <c r="AV4" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX4" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA4" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD4" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF4">
+        <v>1001</v>
+      </c>
+      <c r="BG4" s="4"/>
+      <c r="BH4">
+        <v>1004</v>
+      </c>
+      <c r="BQ4" s="3">
+        <v>901201180204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D5" t="s">
+        <v>191</v>
+      </c>
+      <c r="G5" s="5">
+        <v>32528</v>
+      </c>
+      <c r="H5" t="s">
+        <v>197</v>
+      </c>
+      <c r="J5" t="s">
+        <v>199</v>
+      </c>
+      <c r="K5" t="s">
+        <v>157</v>
+      </c>
+      <c r="AV5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX5" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF5">
+        <v>1001</v>
+      </c>
+      <c r="BG5" s="4"/>
+      <c r="BH5">
+        <v>1004</v>
+      </c>
+      <c r="BQ5" s="3">
+        <v>962201180204</v>
+      </c>
+    </row>
+    <row r="6" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D6" t="s">
+        <v>194</v>
+      </c>
+      <c r="G6" s="5">
+        <v>32833</v>
+      </c>
+      <c r="H6" t="s">
+        <v>154</v>
+      </c>
+      <c r="J6" t="s">
+        <v>156</v>
+      </c>
+      <c r="K6" t="s">
+        <v>157</v>
+      </c>
+      <c r="L6" s="5">
+        <v>32831</v>
+      </c>
+      <c r="N6" t="s">
+        <v>200</v>
+      </c>
+      <c r="O6" t="s">
+        <v>160</v>
+      </c>
+      <c r="P6" s="5">
+        <v>46035</v>
+      </c>
+      <c r="Q6">
+        <v>562</v>
+      </c>
+      <c r="AV6" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX6" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY6" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA6" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB6" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC6" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF6">
+        <v>1001</v>
+      </c>
+      <c r="BG6" s="4"/>
+      <c r="BH6">
+        <v>1004</v>
+      </c>
+      <c r="BQ6" s="3">
+        <v>961001180204</v>
+      </c>
+    </row>
+    <row r="7" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" t="s">
+        <v>196</v>
+      </c>
+      <c r="G7" s="5">
+        <v>36412</v>
+      </c>
+      <c r="H7" t="s">
+        <v>197</v>
+      </c>
+      <c r="J7" t="s">
+        <v>156</v>
+      </c>
+      <c r="K7" t="s">
+        <v>157</v>
+      </c>
+      <c r="L7" s="5">
+        <v>32831</v>
+      </c>
+      <c r="N7" t="s">
+        <v>200</v>
+      </c>
+      <c r="O7" t="s">
+        <v>201</v>
+      </c>
+      <c r="P7" s="5">
+        <v>45691</v>
+      </c>
+      <c r="Q7">
+        <v>123</v>
+      </c>
+      <c r="R7" t="s">
+        <v>164</v>
+      </c>
+      <c r="AV7" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX7" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY7" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA7" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB7" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC7" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD7" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF7">
+        <v>1001</v>
+      </c>
+      <c r="BG7" s="4"/>
+      <c r="BH7">
+        <v>1004</v>
+      </c>
+      <c r="BQ7" s="3">
+        <v>961201180200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>32477</v>
+      </c>
+      <c r="B8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D8" t="s">
+        <v>183</v>
+      </c>
+      <c r="G8" s="5">
+        <v>32835</v>
+      </c>
+      <c r="H8" t="s">
+        <v>154</v>
+      </c>
+      <c r="J8" t="s">
+        <v>198</v>
+      </c>
+      <c r="AV8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX8" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY8" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA8" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB8" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC8" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD8" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF8">
+        <v>1001</v>
+      </c>
+      <c r="BG8" s="4"/>
+      <c r="BH8">
+        <v>1004</v>
+      </c>
+      <c r="BQ8" s="3">
+        <v>761201180204</v>
+      </c>
+    </row>
+    <row r="9" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>32478</v>
+      </c>
+      <c r="B9" t="s">
+        <v>184</v>
+      </c>
+      <c r="D9" t="s">
+        <v>185</v>
+      </c>
+      <c r="G9" s="5">
+        <v>32836</v>
+      </c>
+      <c r="H9" t="s">
+        <v>197</v>
+      </c>
+      <c r="J9" t="s">
+        <v>156</v>
+      </c>
+      <c r="AV9" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW9" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX9" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY9" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA9" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB9" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC9" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD9" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF9">
+        <v>1001</v>
+      </c>
+      <c r="BG9" s="4"/>
+      <c r="BH9">
+        <v>1004</v>
+      </c>
+      <c r="BQ9" s="3">
+        <v>661201180206</v>
+      </c>
+    </row>
+    <row r="10" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>30479</v>
+      </c>
+      <c r="B10" t="s">
+        <v>186</v>
+      </c>
+      <c r="D10" t="s">
+        <v>187</v>
+      </c>
+      <c r="G10" s="5">
+        <v>32837</v>
+      </c>
+      <c r="H10" t="s">
+        <v>197</v>
+      </c>
+      <c r="J10" t="s">
+        <v>156</v>
+      </c>
+      <c r="AV10" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW10" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX10" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY10" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA10" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB10" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC10" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD10" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF10">
+        <v>1001</v>
+      </c>
+      <c r="BG10" s="4"/>
+      <c r="BH10">
+        <v>1004</v>
+      </c>
+      <c r="BQ10" s="3">
+        <v>999201180204</v>
+      </c>
+    </row>
+    <row r="11" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>32479</v>
+      </c>
+      <c r="B11" t="s">
+        <v>188</v>
+      </c>
+      <c r="D11" t="s">
+        <v>189</v>
+      </c>
+      <c r="AV11" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW11" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX11" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY11" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA11" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB11" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC11" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD11" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF11">
+        <v>1001</v>
+      </c>
+      <c r="BG11" s="4"/>
+      <c r="BH11">
+        <v>1004</v>
+      </c>
+      <c r="BQ11" s="3">
+        <v>456781180204</v>
+      </c>
+    </row>
+    <row r="12" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="AV12" t="s">
+        <v>166</v>
+      </c>
+      <c r="AW12" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX12" t="s">
+        <v>168</v>
+      </c>
+      <c r="AY12" t="s">
+        <v>169</v>
+      </c>
+      <c r="BA12" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB12" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC12" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD12" t="s">
+        <v>172</v>
+      </c>
+      <c r="BF12">
+        <v>1001</v>
+      </c>
+      <c r="BG12" s="4"/>
+      <c r="BH12">
+        <v>1004</v>
+      </c>
+      <c r="BQ12" s="3">
+        <v>900200080204</v>
+      </c>
+    </row>
+    <row r="13" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="BG13" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>